<commit_message>
Added in Gas and Electricity cost and usage into Power BI
</commit_message>
<xml_diff>
--- a/Ice Depth Project/BillHistory_Account_Electric.xlsx
+++ b/Ice Depth Project/BillHistory_Account_Electric.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\other-files\school\database_dev\The-Windigo-Data-Team-Summer-2026\Ice Depth Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6CEC30-96A2-499A-AEDF-FEBCE44D093B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DEBDD70-01CA-441F-BF0B-52A4B72FE506}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="690" windowWidth="29040" windowHeight="17520" xr2:uid="{2C695120-188F-48AA-88E0-ADAA39F614CF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{2C695120-188F-48AA-88E0-ADAA39F614CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="41">
   <si>
     <t>Bill date</t>
   </si>
@@ -159,6 +159,9 @@
   </si>
   <si>
     <t>Avg kWh / day</t>
+  </si>
+  <si>
+    <t>Read date</t>
   </si>
 </sst>
 </file>
@@ -546,1207 +549,1254 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2345A3C3-FAC1-44D1-B1DF-D5824D0A5EB0}">
-  <dimension ref="A1:X15"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="22.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" customWidth="1"/>
-    <col min="10" max="10" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="32.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="28.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.85546875" customWidth="1"/>
-    <col min="22" max="22" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="22.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.42578125" customWidth="1"/>
+    <col min="11" max="11" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="28.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.85546875" customWidth="1"/>
+    <col min="23" max="23" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2">
         <v>30</v>
       </c>
-      <c r="C2">
+      <c r="D2">
         <v>1932.48</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>1948.2</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>2451.59</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>749.25</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>60</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>162.47</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>363.51</v>
       </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>19798</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>32470</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>122</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>222</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>61</v>
       </c>
-      <c r="Q2">
+      <c r="R2">
         <v>137</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>32</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>34</v>
       </c>
-      <c r="T2">
-        <f>SUM(C2:I2)</f>
+      <c r="U2">
+        <f>SUM(D2:J2)</f>
         <v>7667.5000000000009</v>
       </c>
-      <c r="U2">
-        <f>SUM(T2, J2:K2)</f>
+      <c r="V2">
+        <f>SUM(U2, K2:L2)</f>
         <v>7667.5000000000009</v>
       </c>
-      <c r="V2" s="2">
-        <f xml:space="preserve"> T2/B2</f>
+      <c r="W2" s="2">
+        <f xml:space="preserve"> U2/C2</f>
         <v>255.58333333333337</v>
       </c>
-      <c r="W2">
-        <f>SUM(L2:M2)</f>
+      <c r="X2">
+        <f>SUM(M2:N2)</f>
         <v>52268</v>
       </c>
-      <c r="X2">
-        <f>W2/B2</f>
+      <c r="Y2">
+        <f>X2/C2</f>
         <v>1742.2666666666667</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
         <v>28</v>
       </c>
-      <c r="C3">
+      <c r="D3">
         <v>2028.43</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>1989</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>2632.44</v>
       </c>
-      <c r="F3">
+      <c r="G3">
         <v>749.25</v>
       </c>
-      <c r="G3">
+      <c r="H3">
         <v>56</v>
       </c>
-      <c r="H3">
+      <c r="I3">
         <v>166.39</v>
       </c>
-      <c r="I3">
+      <c r="J3">
         <v>379.39</v>
       </c>
-      <c r="J3">
+      <c r="K3">
         <v>74.44</v>
       </c>
-      <c r="K3">
+      <c r="L3">
         <v>7814.65</v>
       </c>
-      <c r="L3">
+      <c r="M3">
         <v>20781</v>
       </c>
-      <c r="M3">
+      <c r="N3">
         <v>33150</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>131</v>
       </c>
-      <c r="O3">
+      <c r="P3">
         <v>222</v>
       </c>
-      <c r="P3">
+      <c r="Q3">
         <v>271</v>
       </c>
-      <c r="Q3">
+      <c r="R3">
         <v>9</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>32</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>34</v>
       </c>
-      <c r="T3">
-        <f t="shared" ref="T3:T15" si="0">SUM(C3:I3)</f>
+      <c r="U3">
+        <f t="shared" ref="U3:U15" si="0">SUM(D3:J3)</f>
         <v>8000.9000000000015</v>
       </c>
-      <c r="U3">
-        <f>SUM(T3, J3:K3)</f>
+      <c r="V3">
+        <f>SUM(U3, K3:L3)</f>
         <v>15889.990000000002</v>
       </c>
-      <c r="V3" s="2">
-        <f t="shared" ref="V3:V15" si="1" xml:space="preserve"> T3/B3</f>
+      <c r="W3" s="2">
+        <f t="shared" ref="W3:W15" si="1" xml:space="preserve"> U3/C3</f>
         <v>285.74642857142862</v>
       </c>
-      <c r="W3">
-        <f t="shared" ref="W3:W15" si="2">SUM(L3:M3)</f>
+      <c r="X3">
+        <f t="shared" ref="X3:X15" si="2">SUM(M3:N3)</f>
         <v>53931</v>
       </c>
-      <c r="X3">
-        <f t="shared" ref="X3:X15" si="3">W3/B3</f>
+      <c r="Y3">
+        <f t="shared" ref="Y3:Y15" si="3">X3/C3</f>
         <v>1926.1071428571429</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4">
         <v>33</v>
       </c>
-      <c r="C4">
+      <c r="D4">
         <v>2137.66</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>2184.9</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>2250.64</v>
       </c>
-      <c r="F4">
+      <c r="G4">
         <v>627.75</v>
       </c>
-      <c r="G4">
+      <c r="H4">
         <v>66</v>
       </c>
-      <c r="H4">
+      <c r="I4">
         <v>177.18</v>
       </c>
-      <c r="I4">
+      <c r="J4">
         <v>370.52</v>
       </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
       <c r="K4">
         <v>0</v>
       </c>
       <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>21900</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>36415</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>112</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>186</v>
       </c>
-      <c r="P4">
+      <c r="Q4">
         <v>723</v>
       </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4" t="s">
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s">
         <v>32</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>34</v>
       </c>
-      <c r="T4">
+      <c r="U4">
         <f t="shared" si="0"/>
         <v>7814.65</v>
       </c>
-      <c r="U4">
-        <f t="shared" ref="U4:U15" si="4">SUM(T4, J4:K4)</f>
+      <c r="V4">
+        <f t="shared" ref="V4:V15" si="4">SUM(U4, K4:L4)</f>
         <v>7814.65</v>
       </c>
-      <c r="V4" s="2">
+      <c r="W4" s="2">
         <f t="shared" si="1"/>
         <v>236.80757575757573</v>
       </c>
-      <c r="W4">
+      <c r="X4">
         <f t="shared" si="2"/>
         <v>58315</v>
       </c>
-      <c r="X4">
+      <c r="Y4">
         <f t="shared" si="3"/>
         <v>1767.121212121212</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5">
         <v>29</v>
       </c>
-      <c r="C5">
+      <c r="D5">
         <v>2246.69</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>2230.38</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>2331.02</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>627.75</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>58</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>181.79</v>
       </c>
-      <c r="I5">
+      <c r="J5">
         <v>382.1</v>
       </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
         <v>23017</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>37173</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>116</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>186</v>
       </c>
-      <c r="P5">
+      <c r="Q5">
         <v>839</v>
       </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5" t="s">
         <v>32</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>34</v>
       </c>
-      <c r="T5">
+      <c r="U5">
         <f t="shared" si="0"/>
         <v>8057.7300000000005</v>
       </c>
-      <c r="U5">
+      <c r="V5">
         <f t="shared" si="4"/>
         <v>8057.7300000000005</v>
       </c>
-      <c r="V5" s="2">
+      <c r="W5" s="2">
         <f t="shared" si="1"/>
         <v>277.85275862068966</v>
       </c>
-      <c r="W5">
+      <c r="X5">
         <f t="shared" si="2"/>
         <v>60190</v>
       </c>
-      <c r="X5">
+      <c r="Y5">
         <f t="shared" si="3"/>
         <v>2075.5172413793102</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6">
         <v>27</v>
       </c>
-      <c r="C6">
+      <c r="D6">
         <v>3380.43</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>3367.38</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>3717.58</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>627.75</v>
       </c>
-      <c r="G6">
+      <c r="H6">
         <v>54</v>
       </c>
-      <c r="H6">
+      <c r="I6">
         <v>256.97000000000003</v>
       </c>
-      <c r="I6">
+      <c r="J6">
         <v>568.52</v>
       </c>
-      <c r="J6">
+      <c r="K6">
         <v>84.53</v>
       </c>
-      <c r="K6">
+      <c r="L6">
         <v>8869.6200000000008</v>
       </c>
-      <c r="L6">
+      <c r="M6">
         <v>34632</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>56123</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>185</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>186</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>1404</v>
       </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6" t="s">
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6" t="s">
         <v>32</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>34</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <f t="shared" si="0"/>
         <v>11972.63</v>
       </c>
-      <c r="U6">
+      <c r="V6">
         <f t="shared" si="4"/>
         <v>20926.78</v>
       </c>
-      <c r="V6" s="2">
+      <c r="W6" s="2">
         <f t="shared" si="1"/>
         <v>443.4307407407407</v>
       </c>
-      <c r="W6">
+      <c r="X6">
         <f t="shared" si="2"/>
         <v>90755</v>
       </c>
-      <c r="X6">
+      <c r="Y6">
         <f t="shared" si="3"/>
         <v>3361.2962962962961</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7">
         <v>35</v>
       </c>
-      <c r="C7">
+      <c r="D7">
         <v>2298.6799999999998</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>2687.89</v>
       </c>
-      <c r="E7">
+      <c r="F7">
         <v>2634.61</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>559.94000000000005</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>70</v>
       </c>
-      <c r="H7">
+      <c r="I7">
         <v>124.36</v>
       </c>
-      <c r="I7">
+      <c r="J7">
         <v>417.09</v>
       </c>
-      <c r="J7">
+      <c r="K7">
         <v>77.05</v>
       </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
       <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
         <v>24797</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>47074</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>127</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>168</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>1324</v>
       </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7" t="s">
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7" t="s">
         <v>32</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>34</v>
       </c>
-      <c r="T7">
+      <c r="U7">
         <f t="shared" si="0"/>
         <v>8792.5700000000015</v>
       </c>
-      <c r="U7">
+      <c r="V7">
         <f t="shared" si="4"/>
         <v>8869.6200000000008</v>
       </c>
-      <c r="V7" s="2">
+      <c r="W7" s="2">
         <f t="shared" si="1"/>
         <v>251.21628571428576</v>
       </c>
-      <c r="W7">
+      <c r="X7">
         <f t="shared" si="2"/>
         <v>71871</v>
       </c>
-      <c r="X7">
+      <c r="Y7">
         <f t="shared" si="3"/>
         <v>2053.457142857143</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8">
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8">
         <v>34</v>
       </c>
-      <c r="C8">
+      <c r="D8">
         <v>2196.42</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>2514.67</v>
       </c>
-      <c r="E8">
+      <c r="F8">
         <v>2302.6799999999998</v>
       </c>
-      <c r="F8">
+      <c r="G8">
         <v>555.24</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>68</v>
       </c>
-      <c r="H8">
+      <c r="I8">
         <v>68.16</v>
       </c>
-      <c r="I8">
+      <c r="J8">
         <v>383.57</v>
       </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
       <c r="K8">
         <v>0</v>
       </c>
       <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
         <v>24489</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>45630</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>117</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>168</v>
       </c>
-      <c r="P8">
+      <c r="Q8">
         <v>1092</v>
       </c>
-      <c r="Q8">
-        <v>0</v>
-      </c>
-      <c r="R8" t="s">
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8" t="s">
         <v>32</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>34</v>
       </c>
-      <c r="T8">
+      <c r="U8">
         <f t="shared" si="0"/>
         <v>8088.74</v>
       </c>
-      <c r="U8">
+      <c r="V8">
         <f t="shared" si="4"/>
         <v>8088.74</v>
       </c>
-      <c r="V8" s="2">
+      <c r="W8" s="2">
         <f t="shared" si="1"/>
         <v>237.90411764705883</v>
       </c>
-      <c r="W8">
+      <c r="X8">
         <f t="shared" si="2"/>
         <v>70119</v>
       </c>
-      <c r="X8">
+      <c r="Y8">
         <f t="shared" si="3"/>
         <v>2062.3235294117649</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9">
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9">
         <v>28</v>
       </c>
-      <c r="C9">
+      <c r="D9">
         <v>1772.36</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>1872.91</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>2125.5500000000002</v>
       </c>
-      <c r="F9">
+      <c r="G9">
         <v>555.24</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>56</v>
       </c>
-      <c r="H9">
+      <c r="I9">
         <v>60.59</v>
       </c>
-      <c r="I9">
+      <c r="J9">
         <v>320.45</v>
       </c>
-      <c r="J9">
+      <c r="K9">
         <v>66.59</v>
       </c>
-      <c r="K9">
+      <c r="L9">
         <v>6990.56</v>
       </c>
-      <c r="L9">
+      <c r="M9">
         <v>19761</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>33985</v>
       </c>
-      <c r="N9">
+      <c r="O9">
         <v>108</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>168</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>400</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>3</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>32</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>34</v>
       </c>
-      <c r="T9">
+      <c r="U9">
         <f t="shared" si="0"/>
         <v>6763.0999999999995</v>
       </c>
-      <c r="U9">
+      <c r="V9">
         <f t="shared" si="4"/>
         <v>13820.25</v>
       </c>
-      <c r="V9" s="2">
+      <c r="W9" s="2">
         <f t="shared" si="1"/>
         <v>241.53928571428568</v>
       </c>
-      <c r="W9">
+      <c r="X9">
         <f t="shared" si="2"/>
         <v>53746</v>
       </c>
-      <c r="X9">
+      <c r="Y9">
         <f t="shared" si="3"/>
         <v>1919.5</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10">
+      <c r="B10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10">
         <v>28</v>
       </c>
-      <c r="C10">
+      <c r="D10">
         <v>2103.0500000000002</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>2056.48</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>3267.05</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>555.24</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>56</v>
       </c>
-      <c r="H10">
+      <c r="I10">
         <v>-1378.54</v>
       </c>
-      <c r="I10">
+      <c r="J10">
         <v>331.28</v>
       </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
       <c r="K10">
         <v>0</v>
       </c>
       <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
         <v>23448</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>37316</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>166</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>168</v>
       </c>
-      <c r="P10">
+      <c r="Q10">
         <v>27</v>
       </c>
-      <c r="Q10">
+      <c r="R10">
         <v>128</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>32</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>34</v>
       </c>
-      <c r="T10">
+      <c r="U10">
         <f t="shared" si="0"/>
         <v>6990.56</v>
       </c>
-      <c r="U10">
+      <c r="V10">
         <f t="shared" si="4"/>
         <v>6990.56</v>
       </c>
-      <c r="V10" s="2">
+      <c r="W10" s="2">
         <f t="shared" si="1"/>
         <v>249.66285714285715</v>
       </c>
-      <c r="W10">
+      <c r="X10">
         <f t="shared" si="2"/>
         <v>60764</v>
       </c>
-      <c r="X10">
+      <c r="Y10">
         <f t="shared" si="3"/>
         <v>2170.1428571428573</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11">
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11">
         <v>30</v>
       </c>
-      <c r="C11">
+      <c r="D11">
         <v>2199.02</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>1990.19</v>
       </c>
-      <c r="E11">
+      <c r="F11">
         <v>2755.34</v>
       </c>
-      <c r="F11">
+      <c r="G11">
         <v>518.89</v>
       </c>
-      <c r="G11">
+      <c r="H11">
         <v>60</v>
       </c>
-      <c r="H11">
+      <c r="I11">
         <v>-754.22</v>
       </c>
-      <c r="I11">
+      <c r="J11">
         <v>336.78</v>
       </c>
-      <c r="J11">
+      <c r="K11">
         <v>74.81</v>
       </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
       <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
         <v>24518</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>36113</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>140</v>
       </c>
-      <c r="O11">
+      <c r="P11">
         <v>157</v>
       </c>
-      <c r="P11">
+      <c r="Q11">
         <v>80</v>
       </c>
-      <c r="Q11">
+      <c r="R11">
         <v>103</v>
       </c>
-      <c r="R11" t="s">
+      <c r="S11" t="s">
         <v>32</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>34</v>
       </c>
-      <c r="T11">
+      <c r="U11">
         <f t="shared" si="0"/>
         <v>7106</v>
       </c>
-      <c r="U11">
+      <c r="V11">
         <f t="shared" si="4"/>
         <v>7180.81</v>
       </c>
-      <c r="V11" s="2">
+      <c r="W11" s="2">
         <f t="shared" si="1"/>
         <v>236.86666666666667</v>
       </c>
-      <c r="W11">
+      <c r="X11">
         <f t="shared" si="2"/>
         <v>60631</v>
       </c>
-      <c r="X11">
+      <c r="Y11">
         <f t="shared" si="3"/>
         <v>2021.0333333333333</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12">
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12">
         <v>30</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>2217.85</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>1846.35</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>2775.02</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>518.89</v>
       </c>
-      <c r="G12">
+      <c r="H12">
         <v>60</v>
       </c>
-      <c r="H12">
+      <c r="I12">
         <v>62.84</v>
       </c>
-      <c r="I12">
+      <c r="J12">
         <v>372.36</v>
       </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
       <c r="K12">
         <v>0</v>
       </c>
       <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
         <v>24728</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>33503</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>141</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>157</v>
       </c>
-      <c r="P12">
-        <v>0</v>
-      </c>
       <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
         <v>246</v>
       </c>
-      <c r="R12" t="s">
+      <c r="S12" t="s">
         <v>32</v>
       </c>
-      <c r="S12" t="s">
+      <c r="T12" t="s">
         <v>34</v>
       </c>
-      <c r="T12">
+      <c r="U12">
         <f t="shared" si="0"/>
         <v>7853.3099999999995</v>
       </c>
-      <c r="U12">
+      <c r="V12">
         <f t="shared" si="4"/>
         <v>7853.3099999999995</v>
       </c>
-      <c r="V12" s="2">
+      <c r="W12" s="2">
         <f t="shared" si="1"/>
         <v>261.77699999999999</v>
       </c>
-      <c r="W12">
+      <c r="X12">
         <f t="shared" si="2"/>
         <v>58231</v>
       </c>
-      <c r="X12">
+      <c r="Y12">
         <f t="shared" si="3"/>
         <v>1941.0333333333333</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13">
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13">
         <v>32</v>
       </c>
-      <c r="C13">
+      <c r="D13">
         <v>2135.9699999999998</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>2151.33</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>2873.43</v>
       </c>
-      <c r="F13">
+      <c r="G13">
         <v>518.89</v>
       </c>
-      <c r="G13">
+      <c r="H13">
         <v>64</v>
       </c>
-      <c r="H13">
+      <c r="I13">
         <v>64.55</v>
       </c>
-      <c r="I13">
+      <c r="J13">
         <v>388.75</v>
       </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
         <v>23815</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>39037</v>
       </c>
-      <c r="N13">
+      <c r="O13">
         <v>146</v>
       </c>
-      <c r="O13">
+      <c r="P13">
         <v>157</v>
       </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
       <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
         <v>318</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>32</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>34</v>
       </c>
-      <c r="T13">
+      <c r="U13">
         <f t="shared" si="0"/>
         <v>8196.92</v>
       </c>
-      <c r="U13">
+      <c r="V13">
         <f t="shared" si="4"/>
         <v>8196.92</v>
       </c>
-      <c r="V13" s="2">
+      <c r="W13" s="2">
         <f t="shared" si="1"/>
         <v>256.15375</v>
       </c>
-      <c r="W13">
+      <c r="X13">
         <f t="shared" si="2"/>
         <v>62852</v>
       </c>
-      <c r="X13">
+      <c r="Y13">
         <f t="shared" si="3"/>
         <v>1964.125</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14">
+      <c r="B14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14">
         <v>31</v>
       </c>
-      <c r="C14">
+      <c r="D14">
         <v>1812.37</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>1711</v>
       </c>
-      <c r="E14">
+      <c r="F14">
         <v>2125.5500000000002</v>
       </c>
-      <c r="F14">
+      <c r="G14">
         <v>482.53</v>
       </c>
-      <c r="G14">
+      <c r="H14">
         <v>62</v>
       </c>
-      <c r="H14">
+      <c r="I14">
         <v>58.98</v>
       </c>
-      <c r="I14">
+      <c r="J14">
         <v>310.99</v>
       </c>
-      <c r="J14">
+      <c r="K14">
         <v>59.59</v>
       </c>
-      <c r="K14">
+      <c r="L14">
         <v>6255.27</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>20207</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>31047</v>
       </c>
-      <c r="N14">
+      <c r="O14">
         <v>108</v>
       </c>
-      <c r="O14">
+      <c r="P14">
         <v>146</v>
       </c>
-      <c r="P14">
+      <c r="Q14">
         <v>132</v>
       </c>
-      <c r="Q14">
+      <c r="R14">
         <v>47</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
         <v>32</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>34</v>
       </c>
-      <c r="T14">
+      <c r="U14">
         <f t="shared" si="0"/>
         <v>6563.4199999999992</v>
       </c>
-      <c r="U14">
+      <c r="V14">
         <f t="shared" si="4"/>
         <v>12878.279999999999</v>
       </c>
-      <c r="V14" s="2">
+      <c r="W14" s="2">
         <f t="shared" si="1"/>
         <v>211.72322580645158</v>
       </c>
-      <c r="W14">
+      <c r="X14">
         <f t="shared" si="2"/>
         <v>51254</v>
       </c>
-      <c r="X14">
+      <c r="Y14">
         <f t="shared" si="3"/>
         <v>1653.3548387096773</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15">
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15">
         <v>31</v>
       </c>
-      <c r="C15">
+      <c r="D15">
         <v>1562.13</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>1786.23</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>2007.46</v>
       </c>
-      <c r="F15">
+      <c r="G15">
         <v>482.53</v>
       </c>
-      <c r="G15">
+      <c r="H15">
         <v>62</v>
       </c>
-      <c r="H15">
+      <c r="I15">
         <v>58.61</v>
       </c>
-      <c r="I15">
+      <c r="J15">
         <v>296.31</v>
       </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
         <v>17417</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>32412</v>
       </c>
-      <c r="N15">
+      <c r="O15">
         <v>102</v>
       </c>
-      <c r="O15">
+      <c r="P15">
         <v>146</v>
       </c>
-      <c r="P15">
+      <c r="Q15">
         <v>339</v>
       </c>
-      <c r="Q15">
+      <c r="R15">
         <v>3</v>
       </c>
-      <c r="R15" t="s">
+      <c r="S15" t="s">
         <v>32</v>
       </c>
-      <c r="S15" t="s">
+      <c r="T15" t="s">
         <v>34</v>
       </c>
-      <c r="T15">
+      <c r="U15">
         <f t="shared" si="0"/>
         <v>6255.2699999999995</v>
       </c>
-      <c r="U15">
+      <c r="V15">
         <f t="shared" si="4"/>
         <v>6255.2699999999995</v>
       </c>
-      <c r="V15" s="2">
+      <c r="W15" s="2">
         <f t="shared" si="1"/>
         <v>201.78290322580645</v>
       </c>
-      <c r="W15">
+      <c r="X15">
         <f t="shared" si="2"/>
         <v>49829</v>
       </c>
-      <c r="X15">
+      <c r="Y15">
         <f t="shared" si="3"/>
         <v>1607.3870967741937</v>
       </c>

</xml_diff>